<commit_message>
docs: update C02 status to published in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>リード獲得</t>
+          <t>c02-josler-byoreki-youyaku-template.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update B05 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1184,12 +1184,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>リード獲得</t>
+          <t>b05-josler-shourei-touroku-template.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update keyword list C14 status to published
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -7791,12 +7791,12 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>競合人気テーマ</t>
+          <t>c14-josler-byoreki-youyaku-word-copipe.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update G08 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -3608,12 +3608,12 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>季節更新必要</t>
+          <t>g08-naika-senmoni-nittei.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update keyword list - J02 published
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -4720,12 +4720,12 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>内科ナビ連携</t>
+          <t>j02-byoreki-youyaku-ai-jidou-seisei.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: D01 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1996,10 +1996,14 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>d01-josler-byoreki-youyaku-shoukaki.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
update: add J10 to keyword list as 公開済
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J165"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5086,57 +5086,61 @@
       <c r="J93" s="2" t="n"/>
     </row>
     <row r="94" ht="25" customHeight="1">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>メンタル・生活</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>専攻医 つらい</t>
-        </is>
-      </c>
-      <c r="E94" s="3" t="inlineStr">
-        <is>
-          <t>専攻医がつらい時の乗り越え方｜3年目の壁と対処法</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>共感・解決</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H94" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="I94" s="2" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J94" s="2" t="n"/>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>AI・ツール</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Claude PubMed MCP 医学文献検索</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ClaudeでPubMed論文検索｜MCP連携の設定方法と医学文献の探し方</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>ハウツー</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>j10-claude-pubmed-mcp.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="25" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>K01</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -5151,12 +5155,12 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>後期研修医 きつい</t>
+          <t>専攻医 つらい</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>後期研修医がきつい理由5選｜燃え尽きを防ぐセルフケア</t>
+          <t>専攻医がつらい時の乗り越え方｜3年目の壁と対処法</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -5184,7 +5188,7 @@
     <row r="96" ht="25" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>K02</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5199,12 +5203,12 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>研修医 うつ</t>
+          <t>後期研修医 きつい</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>研修医・専攻医のうつ病リスク｜早期発見と相談先</t>
+          <t>後期研修医がきつい理由5選｜燃え尽きを防ぐセルフケア</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -5214,7 +5218,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
@@ -5232,7 +5236,7 @@
     <row r="97" ht="25" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>K03</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5247,22 +5251,22 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>指導医 合わない</t>
+          <t>研修医 うつ</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>指導医と合わない時の対処法｜ストレスを減らす付き合い方</t>
+          <t>研修医・専攻医のうつ病リスク｜早期発見と相談先</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>問題解決</t>
+          <t>共感・解決</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr">
@@ -5280,7 +5284,7 @@
     <row r="98" ht="25" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>K04</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5295,27 +5299,27 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>医師 ワークライフバランス</t>
+          <t>指導医 合わない</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>医師のワークライフバランス｜専攻医時代の時間管理術</t>
+          <t>指導医と合わない時の対処法｜ストレスを減らす付き合い方</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>問題解決</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -5328,7 +5332,7 @@
     <row r="99" ht="25" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>K05</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5343,17 +5347,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>当直 きつい</t>
+          <t>医師 ワークライフバランス</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>当直がきつい時の対策｜疲労回復と睡眠の取り方</t>
+          <t>医師のワークライフバランス｜専攻医時代の時間管理術</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>問題解決</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -5376,7 +5380,7 @@
     <row r="100" ht="25" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>K06</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5391,17 +5395,17 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>医師 睡眠不足</t>
+          <t>当直 きつい</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>医師の睡眠不足対策｜当直明けの過ごし方とリカバリー法</t>
+          <t>当直がきつい時の対策｜疲労回復と睡眠の取り方</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>問題解決</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5424,42 +5428,42 @@
     <row r="101" ht="25" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>K07</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>バイト・収入</t>
+          <t>メンタル・生活</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>専攻医 バイト いつから</t>
+          <t>医師 睡眠不足</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>専攻医はバイトいつからできる？始め方と注意点</t>
+          <t>医師の睡眠不足対策｜当直明けの過ごし方とリカバリー法</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -5472,7 +5476,7 @@
     <row r="102" ht="25" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5487,17 +5491,17 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>専攻医 バイト 相場</t>
+          <t>専攻医 バイト いつから</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>専攻医のバイト相場｜当直・外来・健診の時給比較</t>
+          <t>専攻医はバイトいつからできる？始め方と注意点</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>比較検討</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5520,7 +5524,7 @@
     <row r="103" ht="25" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5535,12 +5539,12 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>医師 バイト 探し方</t>
+          <t>専攻医 バイト 相場</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>医師のバイトの探し方｜おすすめ求人サイトと選び方</t>
+          <t>専攻医のバイト相場｜当直・外来・健診の時給比較</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -5568,7 +5572,7 @@
     <row r="104" ht="25" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5583,17 +5587,17 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>専攻医 年収</t>
+          <t>医師 バイト 探し方</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>専攻医の年収はいくら？3年目〜5年目のリアルな給与事情</t>
+          <t>医師のバイトの探し方｜おすすめ求人サイトと選び方</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>比較検討</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -5616,7 +5620,7 @@
     <row r="105" ht="25" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -5631,27 +5635,27 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>医師 副業</t>
+          <t>専攻医 年収</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>医師の副業おすすめ｜バイト以外の収入源と注意点</t>
+          <t>専攻医の年収はいくら？3年目〜5年目のリアルな給与事情</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>比較検討</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -5664,42 +5668,42 @@
     <row r="106" ht="25" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>M01</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>税金・節税</t>
+          <t>バイト・収入</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>医師 確定申告</t>
+          <t>医師 副業</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>医師の確定申告ガイド｜バイト収入がある場合の申告方法</t>
+          <t>医師の副業おすすめ｜バイト以外の収入源と注意点</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>比較検討</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H106" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -5712,7 +5716,7 @@
     <row r="107" ht="25" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>M02</t>
+          <t>M01</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5727,17 +5731,17 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>医師 確定申告 いくらから</t>
+          <t>医師 確定申告</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>医師の確定申告はいくらから必要？副業収入の申告基準</t>
+          <t>医師の確定申告ガイド｜バイト収入がある場合の申告方法</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5760,7 +5764,7 @@
     <row r="108" ht="25" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>M03</t>
+          <t>M02</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5775,17 +5779,17 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>勤務医 節税</t>
+          <t>医師 確定申告 いくらから</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>勤務医の節税対策｜iDeCo・ふるさと納税・経費の活用法</t>
+          <t>医師の確定申告はいくらから必要？副業収入の申告基準</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -5808,7 +5812,7 @@
     <row r="109" ht="25" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>M04</t>
+          <t>M03</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -5823,12 +5827,12 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>医師 ふるさと納税</t>
+          <t>勤務医 節税</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>医師のふるさと納税｜年収別おすすめ金額と返礼品</t>
+          <t>勤務医の節税対策｜iDeCo・ふるさと納税・経費の活用法</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -5838,12 +5842,12 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H109" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
@@ -5856,7 +5860,7 @@
     <row r="110" ht="25" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>M05</t>
+          <t>M04</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5871,12 +5875,12 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>医師 iDeCo</t>
+          <t>医師 ふるさと納税</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>医師がiDeCoを始めるメリット｜掛金と節税効果のシミュレーション</t>
+          <t>医師のふるさと納税｜年収別おすすめ金額と返礼品</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -5904,7 +5908,7 @@
     <row r="111" ht="25" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>M06</t>
+          <t>M05</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -5919,17 +5923,17 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>医師 経費</t>
+          <t>医師 iDeCo</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>医師が経費にできるもの｜学会費・書籍・スクラブの扱い</t>
+          <t>医師がiDeCoを始めるメリット｜掛金と節税効果のシミュレーション</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -5952,42 +5956,42 @@
     <row r="112" ht="25" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>N01</t>
+          <t>M06</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>キャリア</t>
+          <t>税金・節税</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>サブスペシャリティ 選び方</t>
+          <t>医師 経費</t>
         </is>
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>サブスペシャリティの選び方｜消化器・循環器・呼吸器の比較</t>
+          <t>医師が経費にできるもの｜学会費・書籍・スクラブの扱い</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>比較検討</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -6000,7 +6004,7 @@
     <row r="113" ht="25" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>N02</t>
+          <t>N01</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -6015,12 +6019,12 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>内科 サブスペ 人気</t>
+          <t>サブスペシャリティ 選び方</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>内科サブスペシャリティ人気ランキング｜志望者数と将来性</t>
+          <t>サブスペシャリティの選び方｜消化器・循環器・呼吸器の比較</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -6048,7 +6052,7 @@
     <row r="114" ht="25" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>N03</t>
+          <t>N02</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -6063,12 +6067,12 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>大学病院 市中病院 どっち</t>
+          <t>内科 サブスペ 人気</t>
         </is>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>大学病院vs市中病院｜専攻医の研修先選びのポイント</t>
+          <t>内科サブスペシャリティ人気ランキング｜志望者数と将来性</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -6096,7 +6100,7 @@
     <row r="115" ht="25" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>N04</t>
+          <t>N03</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -6111,12 +6115,12 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>医局 入るべきか</t>
+          <t>大学病院 市中病院 どっち</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>医局に入るべきか？メリット・デメリットと判断基準</t>
+          <t>大学病院vs市中病院｜専攻医の研修先選びのポイント</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -6144,7 +6148,7 @@
     <row r="116" ht="25" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>N05</t>
+          <t>N04</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -6159,27 +6163,27 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>内科専門医 キャリア</t>
+          <t>医局 入るべきか</t>
         </is>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>内科専門医取得後のキャリアパス｜開業・勤務医・転職の選択肢</t>
+          <t>医局に入るべきか？メリット・デメリットと判断基準</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>比較検討</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -6192,7 +6196,7 @@
     <row r="117" ht="25" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>N06</t>
+          <t>N05</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -6207,12 +6211,12 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>医師 転職 タイミング</t>
+          <t>内科専門医 キャリア</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>医師の転職ベストタイミング｜専門医取得後がおすすめの理由</t>
+          <t>内科専門医取得後のキャリアパス｜開業・勤務医・転職の選択肢</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -6240,7 +6244,7 @@
     <row r="118" ht="25" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>N07</t>
+          <t>N06</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -6255,12 +6259,12 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>内科 開業</t>
+          <t>医師 転職 タイミング</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>内科で開業するには？必要な資金・期間・準備リスト</t>
+          <t>医師の転職ベストタイミング｜専門医取得後がおすすめの理由</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -6288,42 +6292,42 @@
     <row r="119" ht="25" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>O01</t>
+          <t>N07</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>学会・論文</t>
+          <t>キャリア</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>学会発表 初めて</t>
+          <t>内科 開業</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>【初心者向け】学会発表の準備と心構え｜スライド作成のコツ</t>
+          <t>内科で開業するには？必要な資金・期間・準備リスト</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H119" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -6336,7 +6340,7 @@
     <row r="120" ht="25" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>O02</t>
+          <t>O01</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -6351,12 +6355,12 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>学会 抄録 書き方</t>
+          <t>学会発表 初めて</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>学会抄録の書き方｜採択されるためのポイント</t>
+          <t>【初心者向け】学会発表の準備と心構え｜スライド作成のコツ</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -6384,7 +6388,7 @@
     <row r="121" ht="25" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>O03</t>
+          <t>O02</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6399,12 +6403,12 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>症例報告 書き方</t>
+          <t>学会 抄録 書き方</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>症例報告の書き方｜構成・投稿先・採択率を上げるコツ</t>
+          <t>学会抄録の書き方｜採択されるためのポイント</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -6432,7 +6436,7 @@
     <row r="122" ht="25" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>O04</t>
+          <t>O03</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -6447,12 +6451,12 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>英語論文 読み方</t>
+          <t>症例報告 書き方</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>英語論文の効率的な読み方｜Abstract・Methodsの攻略法</t>
+          <t>症例報告の書き方｜構成・投稿先・採択率を上げるコツ</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -6465,9 +6469,9 @@
           <t>中</t>
         </is>
       </c>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
@@ -6480,7 +6484,7 @@
     <row r="123" ht="25" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>O05</t>
+          <t>O04</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -6495,22 +6499,22 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Impact Factor とは</t>
+          <t>英語論文 読み方</t>
         </is>
       </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
-          <t>Impact Factorとは？医師が知るべきジャーナル評価の基礎</t>
+          <t>英語論文の効率的な読み方｜Abstract・Methodsの攻略法</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
@@ -6528,7 +6532,7 @@
     <row r="124" ht="25" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>O06</t>
+          <t>O05</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -6543,17 +6547,17 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>内科学会 総会</t>
+          <t>Impact Factor とは</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>内科学会総会の参加ガイド｜単位取得と効率的な回り方</t>
+          <t>Impact Factorとは？医師が知るべきジャーナル評価の基礎</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -6576,32 +6580,32 @@
     <row r="125" ht="25" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>O06</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>結婚・出産</t>
+          <t>学会・論文</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>O</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>専攻医 結婚</t>
+          <t>内科学会 総会</t>
         </is>
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
-          <t>専攻医で結婚するタイミング｜ベストな時期と両立のコツ</t>
+          <t>内科学会総会の参加ガイド｜単位取得と効率的な回り方</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -6624,7 +6628,7 @@
     <row r="126" ht="25" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -6639,12 +6643,12 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>医師同士 結婚</t>
+          <t>専攻医 結婚</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>医師同士の結婚｜メリット・デメリットと両立の秘訣</t>
+          <t>専攻医で結婚するタイミング｜ベストな時期と両立のコツ</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -6672,7 +6676,7 @@
     <row r="127" ht="25" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -6687,12 +6691,12 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>専攻医 産休</t>
+          <t>医師同士 結婚</t>
         </is>
       </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
-          <t>専攻医の産休・育休｜取得タイミングとJ-OSLERへの影響</t>
+          <t>医師同士の結婚｜メリット・デメリットと両立の秘訣</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -6702,12 +6706,12 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H127" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
@@ -6720,7 +6724,7 @@
     <row r="128" ht="25" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -6735,27 +6739,27 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>医師 育児 両立</t>
+          <t>専攻医 産休</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>医師の育児と仕事の両立｜時短勤務とキャリア継続</t>
+          <t>専攻医の産休・育休｜取得タイミングとJ-OSLERへの影響</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H128" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
@@ -6768,7 +6772,7 @@
     <row r="129" ht="25" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -6783,17 +6787,17 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>女性医師 キャリア</t>
+          <t>医師 育児 両立</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>女性医師のキャリア｜出産・育児を経ての復帰戦略</t>
+          <t>医師の育児と仕事の両立｜時短勤務とキャリア継続</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -6816,32 +6820,32 @@
     <row r="130" ht="25" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Q01</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>サブスペJ-OSLER</t>
+          <t>結婚・出産</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>J-OSLER 消化器</t>
+          <t>女性医師 キャリア</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>J-OSLER消化器内科版の使い方｜連動研修と病歴要約</t>
+          <t>女性医師のキャリア｜出産・育児を経ての復帰戦略</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -6864,7 +6868,7 @@
     <row r="131" ht="25" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Q02</t>
+          <t>Q01</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6879,12 +6883,12 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>J-OSLER 循環器</t>
+          <t>J-OSLER 消化器</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>J-OSLER循環器内科版ガイド｜カテ症例の登録方法</t>
+          <t>J-OSLER消化器内科版の使い方｜連動研修と病歴要約</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -6912,7 +6916,7 @@
     <row r="132" ht="25" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Q03</t>
+          <t>Q02</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6927,12 +6931,12 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>J-OSLER 呼吸器</t>
+          <t>J-OSLER 循環器</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>J-OSLER呼吸器内科版｜25症例の進め方</t>
+          <t>J-OSLER循環器内科版ガイド｜カテ症例の登録方法</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -6960,7 +6964,7 @@
     <row r="133" ht="25" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Q04</t>
+          <t>Q03</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -6975,12 +6979,12 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>J-OSLER 腎臓</t>
+          <t>J-OSLER 呼吸器</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>J-OSLER腎臓内科版｜透析症例の書き方</t>
+          <t>J-OSLER呼吸器内科版｜25症例の進め方</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -7008,7 +7012,7 @@
     <row r="134" ht="25" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Q05</t>
+          <t>Q04</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -7023,27 +7027,27 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>サブスペ専門医 いつ</t>
+          <t>J-OSLER 腎臓</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>サブスペシャリティ専門医はいつ取れる？最短ルートと必要期間</t>
+          <t>J-OSLER腎臓内科版｜透析症例の書き方</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H134" s="5" t="inlineStr">
-        <is>
-          <t>★★</t>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr">
@@ -7056,27 +7060,27 @@
     <row r="135" ht="25" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>Q05</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>サブスペJ-OSLER</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>内科専門医 とは</t>
+          <t>サブスペ専門医 いつ</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>内科専門医とは？認定内科医との違いと取得のメリット</t>
+          <t>サブスペシャリティ専門医はいつ取れる？最短ルートと必要期間</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -7104,7 +7108,7 @@
     <row r="136" ht="25" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -7119,12 +7123,12 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>新専門医制度</t>
+          <t>内科専門医 とは</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>新専門医制度とは？旧制度との違いと移行措置</t>
+          <t>内科専門医とは？認定内科医との違いと取得のメリット</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -7134,12 +7138,12 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H136" s="2" t="inlineStr">
-        <is>
-          <t>★</t>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H136" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr">
@@ -7152,7 +7156,7 @@
     <row r="137" ht="25" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>R03</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -7167,12 +7171,12 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>内科学会 入会</t>
+          <t>新専門医制度</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>内科学会への入会方法｜会費・特典・手続きの流れ</t>
+          <t>新専門医制度とは？旧制度との違いと移行措置</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -7200,7 +7204,7 @@
     <row r="138" ht="25" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>R03</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -7215,17 +7219,17 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>研修手帳</t>
+          <t>内科学会 入会</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>J-OSLER研修手帳の使い方と記入例</t>
+          <t>内科学会への入会方法｜会費・特典・手続きの流れ</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -7248,107 +7252,103 @@
     <row r="139" ht="25" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
         <is>
+          <t>R04</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>研修手帳</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>J-OSLER研修手帳の使い方と記入例</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>ハウツー</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
           <t>R05</t>
         </is>
       </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>EPOC2 使い方</t>
         </is>
       </c>
-      <c r="E139" s="3" t="inlineStr">
+      <c r="E140" s="3" t="inlineStr">
         <is>
           <t>EPOC2の使い方｜初期研修評価システムの入力ガイド</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
+      <c r="F140" s="2" t="inlineStr">
         <is>
           <t>ハウツー</t>
         </is>
       </c>
-      <c r="G139" s="2" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H139" s="2" t="inlineStr">
+      <c r="H140" s="2" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="I139" s="2" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J139" s="2" t="n"/>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>A09</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>J-OSLER基礎</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>J-OSLER 転出 転入</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>J-OSLER施設異動の手続き完全ガイド｜転出・転入申請の流れ</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>問題解決</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>公式FAQで頻出</t>
-        </is>
-      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -7363,12 +7363,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>J-OSLER プログラム変更</t>
+          <t>J-OSLER 転出 転入</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>J-OSLERプログラム変更はできる？移動手続きと注意点</t>
+          <t>J-OSLER施設異動の手続き完全ガイド｜転出・転入申請の流れ</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -7389,13 +7389,18 @@
       <c r="I141" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>公式FAQで頻出</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -7410,22 +7415,22 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>J-OSLER カリキュラム制</t>
+          <t>J-OSLER プログラム変更</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>J-OSLERカリキュラム制とは？対象者・切替条件・単位の数え方</t>
+          <t>J-OSLERプログラム変更はできる？移動手続きと注意点</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>問題解決</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -7436,18 +7441,13 @@
       <c r="I142" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t>産休・留学者向け</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -7462,22 +7462,22 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>J-OSLER 休止 中断</t>
+          <t>J-OSLER カリキュラム制</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>J-OSLER研修の休止・中断ガイド｜復帰時の手続きと注意点</t>
+          <t>J-OSLERカリキュラム制とは？対象者・切替条件・単位の数え方</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>問題解決</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -7488,13 +7488,18 @@
       <c r="I143" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>産休・留学者向け</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -7509,22 +7514,22 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>J-OSLER 連動研修</t>
+          <t>J-OSLER 休止 中断</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>J-OSLER連動研修（並行研修）の進め方｜内科×サブスペの両立</t>
+          <t>J-OSLER研修の休止・中断ガイド｜復帰時の手続きと注意点</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>問題解決</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -7535,18 +7540,13 @@
       <c r="I144" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t>サブスペ志望者向け</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -7561,17 +7561,17 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>J-OSLER 修了認定</t>
+          <t>J-OSLER 連動研修</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>J-OSLER修了認定の流れ｜申請方法と修了見込の手続き</t>
+          <t>J-OSLER連動研修（並行研修）の進め方｜内科×サブスペの両立</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -7587,13 +7587,18 @@
       <c r="I145" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>サブスペ志望者向け</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>A14</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -7608,22 +7613,22 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>J-OSLER 360度評価 自己評価</t>
+          <t>J-OSLER 修了認定</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>J-OSLER自己評価・360度評価の書き方｜半期ごとの手続きまとめ</t>
+          <t>J-OSLER修了認定の流れ｜申請方法と修了見込の手続き</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -7634,18 +7639,13 @@
       <c r="I146" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>忘れがちな手続き</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>A16</t>
+          <t>A15</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -7660,17 +7660,17 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>J-OSLER ヘルプデスク</t>
+          <t>J-OSLER 360度評価 自己評価</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>J-OSLERトラブル時の問い合わせ先まとめ｜ヘルプデスク活用法</t>
+          <t>J-OSLER自己評価・360度評価の書き方｜半期ごとの手続きまとめ</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>問題解決</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -7680,19 +7680,24 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>忘れがちな手続き</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>A17</t>
+          <t>A16</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7707,69 +7712,64 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>J-OSLER プログラム外症例</t>
+          <t>J-OSLER ヘルプデスク</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>J-OSLERプログラム外症例の登録条件｜初期研修・他施設の症例</t>
+          <t>J-OSLERトラブル時の問い合わせ先まとめ｜ヘルプデスク活用法</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>問題解決</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>条件3つを解説</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>A17</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>病歴要約</t>
+          <t>J-OSLER基礎</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>J-OSLER 病歴要約 文字数</t>
+          <t>J-OSLER プログラム外症例</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>J-OSLER病歴要約の文字数・分量ルール｜A4 2枚に収めるコツ</t>
+          <t>J-OSLERプログラム外症例の登録条件｜初期研修・他施設の症例</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>ハウツー</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -7785,13 +7785,18 @@
       <c r="I149" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>条件3つを解説</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -7806,12 +7811,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>J-OSLER 病歴要約 Word コピペ</t>
+          <t>J-OSLER 病歴要約 文字数</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>J-OSLER病歴要約はWordで下書きが正解｜コピペ手順と注意点</t>
+          <t>J-OSLER病歴要約の文字数・分量ルール｜A4 2枚に収めるコツ</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -7826,24 +7831,19 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>公開済</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>c14-josler-byoreki-youyaku-word-copipe.mdx</t>
+          <t>未着手</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -7858,12 +7858,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>J-OSLER 検査結果 単位</t>
+          <t>J-OSLER 病歴要約 Word コピペ</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>J-OSLER検査結果の記載ルール｜単位統一・フォーマットのコツ</t>
+          <t>J-OSLER病歴要約はWordで下書きが正解｜コピペ手順と注意点</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -7878,19 +7878,24 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>c14-josler-byoreki-youyaku-word-copipe.mdx</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -7905,12 +7910,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>J-OSLER 病歴要約 画像</t>
+          <t>J-OSLER 検査結果 単位</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>J-OSLER病歴要約に画像を入れる方法｜レントゲン・CTの扱い</t>
+          <t>J-OSLER検査結果の記載ルール｜単位統一・フォーマットのコツ</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -7920,12 +7925,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -7937,42 +7942,42 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>G12</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>内科専門医試験</t>
+          <t>病歴要約</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>内科専門医試験 CBT 形式</t>
+          <t>J-OSLER 病歴要約 画像</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>内科専門医試験の出題形式｜CBT・問題数・制限時間を解説</t>
+          <t>J-OSLER病歴要約に画像を入れる方法｜レントゲン・CTの扱い</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>ハウツー</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7984,7 +7989,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>G13</t>
+          <t>G12</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -7999,12 +8004,12 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>内科専門医 受験資格 出願</t>
+          <t>内科専門医試験 CBT 形式</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>内科専門医試験の受験資格と出願手続き｜必要書類チェックリスト</t>
+          <t>内科専門医試験の出題形式｜CBT・問題数・制限時間を解説</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -8031,32 +8036,32 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>N08</t>
+          <t>G13</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>キャリア</t>
+          <t>内科専門医試験</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>専攻医 プログラム 選び方</t>
+          <t>内科専門医 受験資格 出願</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>内科専攻医プログラムの選び方｜比較ポイントと先輩の体験談</t>
+          <t>内科専門医試験の受験資格と出願手続き｜必要書類チェックリスト</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>比較検討</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -8066,24 +8071,19 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>初期研修医の入口記事</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>N09</t>
+          <t>N08</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -8098,17 +8098,17 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>内科 やめたい 転科</t>
+          <t>専攻医 プログラム 選び方</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>内科をやめたい？専攻医の転科・キャリアチェンジを考える前に</t>
+          <t>内科専攻医プログラムの選び方｜比較ポイントと先輩の体験談</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>共感・解決</t>
+          <t>比較検討</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8128,81 +8128,86 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>ニーズ大</t>
+          <t>初期研修医の入口記事</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>N09</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>バイト・収入</t>
+          <t>キャリア</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>医師 奨学金 返済</t>
+          <t>内科 やめたい 転科</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>医師の奨学金返済｜地域枠・義務年限と専門研修の両立</t>
+          <t>内科をやめたい？専攻医の転科・キャリアチェンジを考える前に</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>共感・解決</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>ニーズ大</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>メンタル・生活</t>
+          <t>バイト・収入</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>専攻医 当直 回数</t>
+          <t>医師 奨学金 返済</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>専攻医の当直は月何回？回数制限と労働環境の実態</t>
+          <t>医師の奨学金返済｜地域枠・義務年限と専門研修の両立</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -8212,12 +8217,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8229,42 +8234,42 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>M07</t>
+          <t>K08</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>税金・節税</t>
+          <t>メンタル・生活</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>医師 保険 おすすめ</t>
+          <t>専攻医 当直 回数</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>医師におすすめの保険｜勤務医が入るべき保険と不要な保険</t>
+          <t>専攻医の当直は月何回？回数制限と労働環境の実態</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>比較検討</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8276,42 +8281,42 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>A18</t>
+          <t>M07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>J-OSLER基礎</t>
+          <t>税金・節税</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>J-OSLER 学会発表 条件</t>
+          <t>医師 保険 おすすめ</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>J-OSLER学会発表の条件｜2回の実績を確実に満たす方法</t>
+          <t>医師におすすめの保険｜勤務医が入るべき保険と不要な保険</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>情報収集</t>
+          <t>比較検討</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -8323,7 +8328,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>A19</t>
+          <t>A18</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -8338,12 +8343,12 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>J-OSLER 受持期間</t>
+          <t>J-OSLER 学会発表 条件</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>J-OSLER受持期間のルール｜何日以上必要？中央値11日の実態</t>
+          <t>J-OSLER学会発表の条件｜2回の実績を確実に満たす方法</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -8353,12 +8358,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -8370,27 +8375,27 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>R06</t>
+          <t>A19</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>J-OSLER基礎</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>内科専門医 年収 メリット</t>
+          <t>J-OSLER 受持期間</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>内科専門医を取るメリット｜年収・キャリアへの影響を徹底検証</t>
+          <t>J-OSLER受持期間のルール｜何日以上必要？中央値11日の実態</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -8400,12 +8405,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -8417,7 +8422,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>R07</t>
+          <t>R06</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -8432,12 +8437,12 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>研修医 内科 志望動機</t>
+          <t>内科専門医 年収 メリット</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>内科を選んだ理由｜先輩専攻医の志望動機と内科の魅力</t>
+          <t>内科専門医を取るメリット｜年収・キャリアへの影響を徹底検証</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -8447,54 +8452,49 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="J163" t="inlineStr">
-        <is>
-          <t>初期研修医集客</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>A20</t>
+          <t>R07</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>J-OSLER基礎</t>
+          <t>その他</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>R</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>J-OSLER エラー 不具合</t>
+          <t>研修医 内科 志望動機</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>J-OSLERが動かない？エラー・不具合の対処法まとめ</t>
+          <t>内科を選んだ理由｜先輩専攻医の志望動機と内科の魅力</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>問題解決</t>
+          <t>情報収集</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -8510,51 +8510,103 @@
       <c r="I164" t="inlineStr">
         <is>
           <t>未着手</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>初期研修医集客</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>J-OSLER基礎</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>J-OSLER エラー 不具合</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>J-OSLERが動かない？エラー・不具合の対処法まとめ</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>問題解決</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
           <t>R08</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B166" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C166" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr">
+      <c r="D166" t="inlineStr">
         <is>
           <t>ダブルボード 内科</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
+      <c r="E166" t="inlineStr">
         <is>
           <t>ダブルボードとは？内科専門医×他領域の取得方法と条件</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr">
+      <c r="F166" t="inlineStr">
         <is>
           <t>情報収集</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr">
+      <c r="G166" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr">
+      <c r="H166" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr">
+      <c r="I166" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>

</xml_diff>

<commit_message>
update: D05 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -2204,10 +2204,14 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>d05-josler-byoreki-youyaku-jinzou.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="2" t="inlineStr">

</xml_diff>